<commit_message>
members: add Abdullah Mohsin & Hassaan Tayyab; update Aaliyah's info
- Abdullah Mohsin: Undergraduate RA (Apr 2026 - Pres), with photo.
- Hassaan Tayyab: MITACS GRI'26 Intern, photo pending.
- Aaliyah Chang: filled in email, hobbies, and role.
</commit_message>
<xml_diff>
--- a/updates/members/aaliyah-chang/info.xlsx
+++ b/updates/members/aaliyah-chang/info.xlsx
@@ -514,7 +514,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>MASc Student in Electrical and Computer Engineering</t>
+          <t>MASc (Fall 2025 - Pres)</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr"/>
@@ -527,7 +527,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>aaliyah.chang@queensu.ca</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr"/>
@@ -540,7 +540,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Rollerskating, reading, knitting</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr"/>
@@ -568,7 +568,6 @@
           <t>Joined</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
       <c r="C8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
@@ -577,7 +576,6 @@
           <t>Left</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
       <c r="C9" s="3" t="inlineStr"/>
     </row>
   </sheetData>

</xml_diff>